<commit_message>
replace brown belts transformatin
</commit_message>
<xml_diff>
--- a/public/tests/examen ejemplo 2.xlsx
+++ b/public/tests/examen ejemplo 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlan\Desktop\apallzac-tools\public\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1325A81-BF09-4E01-8019-398E2746E6BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A8794D-FAD7-4C08-8D17-E6A66D1CA8F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EAAE7C4-7F0C-41D1-914D-5CF37DDFF1E5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="68">
   <si>
     <t>Escuela</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>Alumno 50</t>
+  </si>
+  <si>
+    <t>Café 1er grado</t>
   </si>
 </sst>
 </file>
@@ -696,7 +699,7 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="E5" t="s">
         <v>16</v>

</xml_diff>